<commit_message>
data(it): 엑셀 업로드 처리 — Global Request 반영
</commit_message>
<xml_diff>
--- a/it/_upload/IT_product_status.xlsx
+++ b/it/_upload/IT_product_status.xlsx
@@ -5071,7 +5071,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>[WB] In progress</t>
+          <t>[QA] QA review</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -8239,7 +8239,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 09:25</t>
+          <t>2026-10-07 14:44</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8273,7 +8273,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>raw-data-20261003.xlsb</t>
+          <t>raw-data-20261007.xlsb</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>